<commit_message>
commit 12072026 work on mortality quality testing
</commit_message>
<xml_diff>
--- a/inst/resources/variable_schema_data_household_template.xlsx
+++ b/inst/resources/variable_schema_data_household_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R Projects\SaeedR1987\public_health_resources\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R Projects\Positron\public_health_resources\inst\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4D9823B-F4A3-4D13-948C-63174DA3034F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42A92279-E358-469F-8E42-9A8931ECE687}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42179,59 +42179,59 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B762:B813">
+    <cfRule type="duplicateValues" dxfId="17" priority="30"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C756:C759 C762:C764">
-    <cfRule type="duplicateValues" dxfId="17" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C766:C768">
-    <cfRule type="duplicateValues" dxfId="16" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="22"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C770:C772 C774:C779">
+    <cfRule type="duplicateValues" dxfId="14" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J762:J773">
-    <cfRule type="duplicateValues" dxfId="15" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="19"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J774:J776">
+    <cfRule type="duplicateValues" dxfId="12" priority="34"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J777:J779">
+    <cfRule type="duplicateValues" dxfId="11" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J780:J781">
-    <cfRule type="duplicateValues" dxfId="14" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J795:J797 J800">
-    <cfRule type="duplicateValues" dxfId="13" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J798">
-    <cfRule type="duplicateValues" dxfId="12" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J799">
-    <cfRule type="duplicateValues" dxfId="11" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J801:J802">
-    <cfRule type="duplicateValues" dxfId="10" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J804">
-    <cfRule type="duplicateValues" dxfId="9" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J805">
-    <cfRule type="duplicateValues" dxfId="8" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J807">
-    <cfRule type="duplicateValues" dxfId="7" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J808">
-    <cfRule type="duplicateValues" dxfId="6" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J810:J813">
-    <cfRule type="duplicateValues" dxfId="5" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="P742:P754">
-    <cfRule type="duplicateValues" dxfId="4" priority="27"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B762:B813">
-    <cfRule type="duplicateValues" dxfId="3" priority="30"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C770:C772 C774:C779">
-    <cfRule type="duplicateValues" dxfId="2" priority="32"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J774:J776">
-    <cfRule type="duplicateValues" dxfId="1" priority="34"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J777:J779">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="27"/>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>